<commit_message>
Apply CJ072501 Total CBD correction (26.20 -> 0.09, paper-verified) and Sheets decimal-comma fix
- CJ072501/ППК25367: extraction filed the Δ9-THCA component line (26.20)
  as Total CBD; QC eye-checked the paper certificate — Вкупно CBD = 0.09.
  Correction added to the CORRECTIONS overlay with evidence note; register,
  dossier and workbook rebuilt.
- register_sheets.csv / dossier_sheets.csv: renditions for Google Sheets
  upload with bare decimal-comma numerics normalized to decimal points —
  Sheets' CSV import parses 0,016-style values with the comma as a
  thousands separator (0,016 -> 16), which had corrupted the metals and
  mycotoxin columns in the first uploaded Sheet. Values unchanged in
  substance; separator only.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DyBhj47i7bhaCyNMB1iwdv
</commit_message>
<xml_diff>
--- a/deliverables/qc_register/PP_Batch_QC_Testing_Results_Register.xlsx
+++ b/deliverables/qc_register/PP_Batch_QC_Testing_Results_Register.xlsx
@@ -4750,8 +4750,8 @@
       <c r="L33" s="10" t="n">
         <v>23.7</v>
       </c>
-      <c r="M33" s="10" t="n">
-        <v>26.2</v>
+      <c r="M33" s="14" t="n">
+        <v>0.09</v>
       </c>
       <c r="N33" s="11" t="inlineStr">
         <is>
@@ -22772,8 +22772,8 @@
         <is>
           <t>627-1128-25 · 02.07.2025 · IJZ-MB
 197-11-K-26 · 07.08.2026 · FHM
+QCCoA 001 · 10.07.2025 · PP
 ППК25174 · 10.07.2025 · CNP
-QCCoA 001 · 10.07.2025 · PP
 197-11-M-26 · 10.08.2026 · FHM
 QCCoA 001 · 17.07.2025 · PP
 3176-2025 · 26.06.2025 · IJZ</t>
@@ -22975,8 +22975,8 @@
       <c r="F19" s="22" t="inlineStr">
         <is>
           <t>QCCoA 001v02 · 21.01.2026 · PP
+3638-2025 · 28.07.2025 · IJZ
 ППК25211 · 28.07.2025 · CNP
-3638-2025 · 28.07.2025 · IJZ
 767-1376-25 · 29.07.2025 · IJZ-MB</t>
         </is>
       </c>
@@ -23620,8 +23620,8 @@
       <c r="F36" s="22" t="inlineStr">
         <is>
           <t>1226-2192-25 · 05.12.2025 · IJZ-MB
+ППК25380 · 12.12.2025 · CNP
 5888-2025 · 12.12.2025 · IJZ
-ППК25380 · 12.12.2025 · CNP
 QCCoA 001v02 · 21.01.2026 · PP</t>
         </is>
       </c>
@@ -24107,8 +24107,8 @@
       </c>
       <c r="F49" s="22" t="inlineStr">
         <is>
-          <t>100-1-K-26 · 09.04.2026 · FHM
-100-1-LoD-26 · 09.04.2026 · FHM</t>
+          <t>100-1-LoD-26 · 09.04.2026 · FHM
+100-1-K-26 · 09.04.2026 · FHM</t>
         </is>
       </c>
       <c r="G49" s="22" t="inlineStr">
@@ -26274,7 +26274,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -26896,90 +26896,112 @@
     <row r="34">
       <c r="A34" s="28" t="inlineStr">
         <is>
+          <t>CJ072501</t>
+        </is>
+      </c>
+      <c r="B34" s="28" t="inlineStr">
+        <is>
+          <t>Total CBD</t>
+        </is>
+      </c>
+      <c r="C34" s="29" t="inlineStr">
+        <is>
+          <t>0.09</t>
+        </is>
+      </c>
+      <c r="D34" s="30" t="inlineStr">
+        <is>
+          <t>extraction row misassignment (took Δ9-THCA 26.20); 0.09 confirmed on paper original by QC</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="28" t="inlineStr">
+        <is>
           <t>AB092501</t>
         </is>
       </c>
-      <c r="B34" s="28" t="inlineStr">
+      <c r="B35" s="28" t="inlineStr">
         <is>
           <t>Total Δ9-THC</t>
         </is>
       </c>
-      <c r="C34" s="29" t="inlineStr">
+      <c r="C35" s="29" t="inlineStr">
         <is>
           <t>16.93</t>
         </is>
       </c>
-      <c r="D34" s="30" t="inlineStr">
+      <c r="D35" s="30" t="inlineStr">
         <is>
           <t>extraction line-pick error, corrected from certificate text</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="18" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="18" t="inlineStr">
         <is>
           <t>D — Batches in the database but NOT in the prior Batch-Release register</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="31" t="inlineStr">
-        <is>
-          <t>GG1024</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="31" t="inlineStr">
         <is>
-          <t>OMP1024_01</t>
+          <t>GG1024</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="31" t="inlineStr">
         <is>
-          <t>BSS1024_01/1</t>
+          <t>OMP1024_01</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="31" t="inlineStr">
         <is>
-          <t>CJ052501/01</t>
+          <t>BSS1024_01/1</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="31" t="inlineStr">
         <is>
-          <t>CJ052501/02</t>
+          <t>CJ052501/01</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="31" t="inlineStr">
         <is>
-          <t>FB012601_1</t>
+          <t>CJ052501/02</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="31" t="inlineStr">
         <is>
-          <t>GG012601*</t>
+          <t>FB012601_1</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="31" t="inlineStr">
         <is>
-          <t>JD012601*</t>
+          <t>GG012601*</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="31" t="inlineStr">
+        <is>
+          <t>JD012601*</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="31" t="inlineStr">
         <is>
           <t>JD112501*</t>
         </is>

</xml_diff>

<commit_message>
Backfill P-numbers from owner tranche sheet; full Drive-tree completeness sweep
- P-numbers backfilled per PP-TH-VER mapping confirmed by the owner:
  JD112501 -> P060212, JD012603/02 -> P060412, JD012603/02V -> P060422;
  Section 4 no-certificate list annotated with the newly supplied P-numbers
  (ACC102501/P060122, CC012603/P060372, CF102501/P060132,
  JD012603-01/P060362, PUM102501/P060112)
- Completeness sweep of the QC_eCoA Drive tree: eCoA_DATABASE folder is a
  perfect 291<->291 id match with the database (0 new, 0 missing, 0 renamed);
  SS_eCoA_DATABASE holds 10 renamed copies of the already-ingested stability
  certificates; WATER_TESTING holds 261 water reports (separate scope)
- 48-value THC check vs database: 39 exact, 3 known discrepancies
  (BSS052501 NGP paper, KC102501 digit swap, PM112501 13.00), 5 batches
  genuinely without certificates

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DyBhj47i7bhaCyNMB1iwdv
</commit_message>
<xml_diff>
--- a/deliverables/qc_register/PP_Batch_QC_Testing_Results_Register.xlsx
+++ b/deliverables/qc_register/PP_Batch_QC_Testing_Results_Register.xlsx
@@ -9582,7 +9582,11 @@
           <t>JD112501</t>
         </is>
       </c>
-      <c r="E67" s="6" t="n"/>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>P060212</t>
+        </is>
+      </c>
       <c r="F67" s="6" t="inlineStr">
         <is>
           <t>Jelly Donutz</t>
@@ -10422,7 +10426,11 @@
           <t>JD012603_02</t>
         </is>
       </c>
-      <c r="E73" s="6" t="n"/>
+      <c r="E73" s="6" t="inlineStr">
+        <is>
+          <t>P060412</t>
+        </is>
+      </c>
       <c r="F73" s="6" t="inlineStr">
         <is>
           <t>JellyDonutz</t>
@@ -10558,7 +10566,11 @@
           <t>JD012603_02V</t>
         </is>
       </c>
-      <c r="E74" s="6" t="n"/>
+      <c r="E74" s="6" t="inlineStr">
+        <is>
+          <t>P060422</t>
+        </is>
+      </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
           <t>JellyDonutz</t>
@@ -19379,7 +19391,11 @@
           <t>JD112501</t>
         </is>
       </c>
-      <c r="B64" s="19" t="n"/>
+      <c r="B64" s="19" t="inlineStr">
+        <is>
+          <t>P060212</t>
+        </is>
+      </c>
       <c r="C64" s="20" t="inlineStr">
         <is>
           <t>197-15-K-26, 07.08.2026, FHM</t>
@@ -20069,7 +20085,11 @@
           <t>JD012603_02</t>
         </is>
       </c>
-      <c r="B70" s="19" t="n"/>
+      <c r="B70" s="19" t="inlineStr">
+        <is>
+          <t>P060412</t>
+        </is>
+      </c>
       <c r="C70" s="20" t="inlineStr">
         <is>
           <t>ППК26113, 30.06.2026, CNP</t>
@@ -20182,7 +20202,11 @@
           <t>JD012603_02V</t>
         </is>
       </c>
-      <c r="B71" s="19" t="n"/>
+      <c r="B71" s="19" t="inlineStr">
+        <is>
+          <t>P060422</t>
+        </is>
+      </c>
       <c r="C71" s="20" t="inlineStr">
         <is>
           <t>ППК26111, 30.06.2026, CNP</t>
@@ -23005,8 +23029,8 @@
       <c r="F13" s="22" t="inlineStr">
         <is>
           <t>QCCoA 001 · 10.07.2025 · PP
+ППК25140 · 22.05.2025 · CNP
 472-0863-25 · 22.05.2025 · IJZ-MB
-ППК25140 · 22.05.2025 · CNP
 2472-2025 · 30.05.2025 · IJZ</t>
         </is>
       </c>
@@ -23044,8 +23068,8 @@
         <is>
           <t>627-1128-25 · 02.07.2025 · IJZ-MB
 197-11-K-26 · 07.08.2026 · FHM
+QCCoA 001 · 10.07.2025 · PP
 ППК25174 · 10.07.2025 · CNP
-QCCoA 001 · 10.07.2025 · PP
 197-11-M-26 · 10.08.2026 · FHM
 QCCoA 001 · 17.07.2025 · PP
 3176-2025 · 26.06.2025 · IJZ</t>
@@ -23393,8 +23417,8 @@
       <c r="F23" s="22" t="inlineStr">
         <is>
           <t>4349-2025 · 15.09.2025 · IJZ
+ППК25281 · 17.09.2025 · CNP
 947-1685-25 · 17.09.2025 · IJZ-MB
-ППК25281 · 17.09.2025 · CNP
 QCCoA 001v02 · 21.01.2026 · PP</t>
         </is>
       </c>
@@ -23628,8 +23652,8 @@
       <c r="F29" s="22" t="inlineStr">
         <is>
           <t>5661-2025 · 01.12.2025 · IJZ
+QCCoA 001v02 · 04.12.2025 · PP
 276-31-M-25 · 04.12.2025 · FHM
-QCCoA 001v02 · 04.12.2025 · PP
 10802_2845-2 EN · 17.11.2025 · DFL
 1157-2058-25 · 24.11.2025 · IJZ-MB</t>
         </is>
@@ -23817,8 +23841,8 @@
       <c r="F34" s="22" t="inlineStr">
         <is>
           <t>1228-2194-25 · 05.12.2025 · IJZ-MB
+5886-2025 · 12.12.2025 · IJZ
 ППК25378 · 12.12.2025 · CNP
-5886-2025 · 12.12.2025 · IJZ
 QCCoA 001v02 · 21.01.2026 · PP</t>
         </is>
       </c>
@@ -23933,8 +23957,8 @@
           <t>1227-2193-25 · 05.12.2025 · IJZ-MB
 197-12-K-26 · 07.08.2026 · FHM
 197-12-M-26 · 10.08.2026 · FHM
+5889-2025 · 12.12.2025 · IJZ
 ППК25381 · 12.12.2025 · CNP
-5889-2025 · 12.12.2025 · IJZ
 QCCoA 001v02 · 21.01.2026 · PP</t>
         </is>
       </c>
@@ -24888,7 +24912,11 @@
           <t>JD112501</t>
         </is>
       </c>
-      <c r="D64" s="22" t="n"/>
+      <c r="D64" s="22" t="inlineStr">
+        <is>
+          <t>P060212</t>
+        </is>
+      </c>
       <c r="E64" s="22" t="inlineStr">
         <is>
           <t>Jelly Donutz</t>
@@ -25085,7 +25113,11 @@
           <t>JD012603_02</t>
         </is>
       </c>
-      <c r="D70" s="22" t="n"/>
+      <c r="D70" s="22" t="inlineStr">
+        <is>
+          <t>P060412</t>
+        </is>
+      </c>
       <c r="E70" s="22" t="inlineStr">
         <is>
           <t>JellyDonutz</t>
@@ -25112,7 +25144,11 @@
           <t>JD012603_02V</t>
         </is>
       </c>
-      <c r="D71" s="22" t="n"/>
+      <c r="D71" s="22" t="inlineStr">
+        <is>
+          <t>P060422</t>
+        </is>
+      </c>
       <c r="E71" s="22" t="inlineStr">
         <is>
           <t>JellyDonutz</t>

</xml_diff>

<commit_message>
Tranche 1/2/3 full THC audit: 69/69 certified register values confirmed correct
Audited every Total THC result from every certificate for all Tranche 1-3
batches against the register:
- 67 rows match the CoQ-forming rule directly; 2 rows (OMP1024_01 15.38,
  GG1024_02 15.95) match via the documented certificate-anomaly corrections
  (still flagged VERIFY ON PAPER ORIGINAL); 8 batches pending (no eCoA yet,
  5 of them sampled 12.08.2026)
- Identity resolution from the audit: the tranche sheet's plain GG012601
  (P060302, 15.35) and JD012601 (P060312, 18.16) are exactly the certified
  milled-presentation batches GG012601*/JD012601* (certificates print
  серија GG012601*/JD012601*) — P-numbers and strains backfilled, Section 4
  no-certificate list reduced to 8 entries

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DyBhj47i7bhaCyNMB1iwdv
</commit_message>
<xml_diff>
--- a/deliverables/qc_register/PP_Batch_QC_Testing_Results_Register.xlsx
+++ b/deliverables/qc_register/PP_Batch_QC_Testing_Results_Register.xlsx
@@ -9196,8 +9196,16 @@
           <t>GG012601*</t>
         </is>
       </c>
-      <c r="E64" s="6" t="n"/>
-      <c r="F64" s="6" t="n"/>
+      <c r="E64" s="6" t="inlineStr">
+        <is>
+          <t>P060302</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>Gorilla Glue</t>
+        </is>
+      </c>
       <c r="G64" s="6" t="n"/>
       <c r="H64" s="6" t="n"/>
       <c r="I64" s="6" t="inlineStr">
@@ -9460,8 +9468,16 @@
           <t>JD012601*</t>
         </is>
       </c>
-      <c r="E66" s="6" t="n"/>
-      <c r="F66" s="6" t="n"/>
+      <c r="E66" s="6" t="inlineStr">
+        <is>
+          <t>P060312</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="inlineStr">
+        <is>
+          <t>Jelly Donutz</t>
+        </is>
+      </c>
       <c r="G66" s="6" t="n"/>
       <c r="H66" s="6" t="n"/>
       <c r="I66" s="6" t="inlineStr">
@@ -9717,7 +9733,11 @@
         </is>
       </c>
       <c r="E68" s="6" t="n"/>
-      <c r="F68" s="6" t="n"/>
+      <c r="F68" s="6" t="inlineStr">
+        <is>
+          <t>Jelly Donutz</t>
+        </is>
+      </c>
       <c r="G68" s="6" t="n"/>
       <c r="H68" s="6" t="n"/>
       <c r="I68" s="6" t="inlineStr">
@@ -19048,7 +19068,11 @@
           <t>GG012601*</t>
         </is>
       </c>
-      <c r="B61" s="19" t="n"/>
+      <c r="B61" s="19" t="inlineStr">
+        <is>
+          <t>P060302</t>
+        </is>
+      </c>
       <c r="C61" s="20" t="inlineStr">
         <is>
           <t>ППК26062, 11.05.2026, CNP</t>
@@ -19278,7 +19302,11 @@
           <t>JD012601*</t>
         </is>
       </c>
-      <c r="B63" s="19" t="n"/>
+      <c r="B63" s="19" t="inlineStr">
+        <is>
+          <t>P060312</t>
+        </is>
+      </c>
       <c r="C63" s="20" t="inlineStr">
         <is>
           <t>ППК26064, 11.05.2026, CNP</t>
@@ -23068,8 +23096,8 @@
         <is>
           <t>627-1128-25 · 02.07.2025 · IJZ-MB
 197-11-K-26 · 07.08.2026 · FHM
+ППК25174 · 10.07.2025 · CNP
 QCCoA 001 · 10.07.2025 · PP
-ППК25174 · 10.07.2025 · CNP
 197-11-M-26 · 10.08.2026 · FHM
 QCCoA 001 · 17.07.2025 · PP
 3176-2025 · 26.06.2025 · IJZ</t>
@@ -23309,8 +23337,8 @@
       <c r="F20" s="22" t="inlineStr">
         <is>
           <t>QCCoA 001v02 · 21.01.2026 · PP
+3636-2025 · 28.07.2025 · IJZ
 ППК25210 · 28.07.2025 · CNP
-3636-2025 · 28.07.2025 · IJZ
 766-1375-25 · 29.07.2025 · IJZ-MB</t>
         </is>
       </c>
@@ -23417,8 +23445,8 @@
       <c r="F23" s="22" t="inlineStr">
         <is>
           <t>4349-2025 · 15.09.2025 · IJZ
+947-1685-25 · 17.09.2025 · IJZ-MB
 ППК25281 · 17.09.2025 · CNP
-947-1685-25 · 17.09.2025 · IJZ-MB
 QCCoA 001v02 · 21.01.2026 · PP</t>
         </is>
       </c>
@@ -23652,8 +23680,8 @@
       <c r="F29" s="22" t="inlineStr">
         <is>
           <t>5661-2025 · 01.12.2025 · IJZ
+276-31-M-25 · 04.12.2025 · FHM
 QCCoA 001v02 · 04.12.2025 · PP
-276-31-M-25 · 04.12.2025 · FHM
 10802_2845-2 EN · 17.11.2025 · DFL
 1157-2058-25 · 24.11.2025 · IJZ-MB</t>
         </is>
@@ -23841,8 +23869,8 @@
       <c r="F34" s="22" t="inlineStr">
         <is>
           <t>1228-2194-25 · 05.12.2025 · IJZ-MB
+ППК25378 · 12.12.2025 · CNP
 5886-2025 · 12.12.2025 · IJZ
-ППК25378 · 12.12.2025 · CNP
 QCCoA 001v02 · 21.01.2026 · PP</t>
         </is>
       </c>
@@ -23917,8 +23945,8 @@
       <c r="F36" s="22" t="inlineStr">
         <is>
           <t>1226-2192-25 · 05.12.2025 · IJZ-MB
+5888-2025 · 12.12.2025 · IJZ
 ППК25380 · 12.12.2025 · CNP
-5888-2025 · 12.12.2025 · IJZ
 QCCoA 001v02 · 21.01.2026 · PP</t>
         </is>
       </c>
@@ -23957,8 +23985,8 @@
           <t>1227-2193-25 · 05.12.2025 · IJZ-MB
 197-12-K-26 · 07.08.2026 · FHM
 197-12-M-26 · 10.08.2026 · FHM
+ППК25381 · 12.12.2025 · CNP
 5889-2025 · 12.12.2025 · IJZ
-ППК25381 · 12.12.2025 · CNP
 QCCoA 001v02 · 21.01.2026 · PP</t>
         </is>
       </c>
@@ -24404,8 +24432,8 @@
       </c>
       <c r="F49" s="22" t="inlineStr">
         <is>
-          <t>100-1-K-26 · 09.04.2026 · FHM
-100-1-LoD-26 · 09.04.2026 · FHM</t>
+          <t>100-1-LoD-26 · 09.04.2026 · FHM
+100-1-K-26 · 09.04.2026 · FHM</t>
         </is>
       </c>
       <c r="G49" s="22" t="inlineStr">
@@ -24825,8 +24853,16 @@
           <t>GG012601*</t>
         </is>
       </c>
-      <c r="D61" s="22" t="n"/>
-      <c r="E61" s="22" t="n"/>
+      <c r="D61" s="22" t="inlineStr">
+        <is>
+          <t>P060302</t>
+        </is>
+      </c>
+      <c r="E61" s="22" t="inlineStr">
+        <is>
+          <t>Gorilla Glue</t>
+        </is>
+      </c>
       <c r="F61" s="22" t="inlineStr">
         <is>
           <t>ППК26062 · 11.05.2026 · CNP
@@ -24887,8 +24923,16 @@
           <t>JD012601*</t>
         </is>
       </c>
-      <c r="D63" s="22" t="n"/>
-      <c r="E63" s="22" t="n"/>
+      <c r="D63" s="22" t="inlineStr">
+        <is>
+          <t>P060312</t>
+        </is>
+      </c>
+      <c r="E63" s="22" t="inlineStr">
+        <is>
+          <t>Jelly Donutz</t>
+        </is>
+      </c>
       <c r="F63" s="22" t="inlineStr">
         <is>
           <t>ППК26064 · 11.05.2026 · CNP
@@ -24949,7 +24993,11 @@
         </is>
       </c>
       <c r="D65" s="22" t="n"/>
-      <c r="E65" s="22" t="n"/>
+      <c r="E65" s="22" t="inlineStr">
+        <is>
+          <t>Jelly Donutz</t>
+        </is>
+      </c>
       <c r="F65" s="22" t="inlineStr">
         <is>
           <t>ППК26065 · 11.05.2026 · CNP

</xml_diff>